<commit_message>
feat(calculators): first test case for beef pasture passing
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.1-beef.xlsx
+++ b/packages/calculators/src/modules/test/4.1-beef.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{D7C6FCB2-875D-AA46-9D2D-92010A8D90F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{B52FBB0C-CCFB-6442-BDD1-71F841E20C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2500" yWindow="880" windowWidth="45460" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51220" yWindow="11700" windowWidth="28800" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4.2.1 methane" sheetId="2" r:id="rId1"/>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="AE11">
         <f>SUM(Q11:R50)</f>
-        <v>516.07877126485812</v>
+        <v>518.72416560985539</v>
       </c>
       <c r="AF11">
         <f>$AS$8</f>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="AG11">
         <f>AE11 * AF11 * 10^-3</f>
-        <v>14.450205595416028</v>
+        <v>14.524276637075952</v>
       </c>
     </row>
     <row r="12" spans="1:53" x14ac:dyDescent="0.2">
@@ -2119,38 +2119,38 @@
         <v>0.3</v>
       </c>
       <c r="J27">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="K27">
         <v>1.3</v>
       </c>
       <c r="L27">
         <f>(J27*K27)+(1 - J27)</f>
-        <v>1.21</v>
+        <v>1.3</v>
       </c>
       <c r="M27">
-        <f t="shared" si="0"/>
-        <v>9.309296640996001</v>
+        <f>(1.185 + 0.00454 * H27 - 0.0000026 * H27^2 + 0.315 * I27)^2 * L27</f>
+        <v>10.001723663880002</v>
       </c>
       <c r="N27">
         <f>(M27 * (1 -S$11) + (0.04 * M27)) * ( 1 - AD$11 )</f>
-        <v>3.8317064974339536</v>
+        <v>4.1167094600530074</v>
       </c>
       <c r="O27">
         <f t="shared" si="1"/>
-        <v>1.8027044885303512E-4</v>
+        <v>1.9367899463549227E-4</v>
       </c>
       <c r="P27">
         <f t="shared" si="2"/>
-        <v>2.1583064698294891E-3</v>
+        <v>2.3188416618002772E-3</v>
       </c>
       <c r="Q27">
         <f t="shared" si="3"/>
-        <v>1.6449678457839456</v>
+        <v>1.7673208260488671</v>
       </c>
       <c r="R27">
         <f t="shared" si="4"/>
-        <v>19.694546537194089</v>
+        <v>21.159430163927528</v>
       </c>
       <c r="BB27" s="2"/>
       <c r="BC27" s="2"/>
@@ -2336,38 +2336,38 @@
         <v>0.3</v>
       </c>
       <c r="J31">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="K31">
         <v>1.3</v>
       </c>
       <c r="L31">
         <f t="shared" si="5"/>
-        <v>1.1800000000000002</v>
+        <v>1.3</v>
       </c>
       <c r="M31">
         <f t="shared" si="0"/>
-        <v>9.0784876333680025</v>
+        <v>10.001723663880002</v>
       </c>
       <c r="N31">
         <f>(M31 * (1 -S$11) + (0.04 * M31)) * ( 1 - AD$11 )</f>
-        <v>3.7367055098942692</v>
+        <v>4.1167094600530074</v>
       </c>
       <c r="O31">
         <f t="shared" si="1"/>
-        <v>1.7580093359221608E-4</v>
+        <v>1.9367899463549227E-4</v>
       </c>
       <c r="P31">
         <f t="shared" si="2"/>
-        <v>2.1047947391725596E-3</v>
+        <v>2.3188416618002772E-3</v>
       </c>
       <c r="Q31">
         <f t="shared" si="3"/>
-        <v>0.80209175951448586</v>
+        <v>0.88366041302443354</v>
       </c>
       <c r="R31">
         <f t="shared" si="4"/>
-        <v>9.6031259974748036</v>
+        <v>10.579715081963764</v>
       </c>
       <c r="BB31" s="2"/>
       <c r="BC31" s="2"/>

</xml_diff>

<commit_message>
feat(calculators): finished json file for beef pasture n2o
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.1-beef.xlsx
+++ b/packages/calculators/src/modules/test/4.1-beef.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{F3CF0DB7-189F-CB48-9787-EEC338E85ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{8FB9131E-94CA-3642-A0E7-6203DA3A4994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2920" yWindow="600" windowWidth="45460" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51080" yWindow="10420" windowWidth="28800" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4.2.1 methane" sheetId="2" r:id="rId1"/>

</xml_diff>